<commit_message>
control de ajustes en fichas
</commit_message>
<xml_diff>
--- a/programas/salidas/Base_resultados_PPDJ_python.xlsx
+++ b/programas/salidas/Base_resultados_PPDJ_python.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB37"/>
+  <dimension ref="A1:AC37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,125 +446,130 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Nuevo (2025)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Esperado</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Nombre indicador</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Indicador tipo</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Sector líder</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Tipo de anualización</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Fecha inicio</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Fecha fin</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Valor_2020</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Meta_2020</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Diff_2020</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Valor_2021</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Meta_2021</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Diff_2021</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Valor_2022</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Meta_2022</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Diff_2022</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Valor_2023</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Meta_2023</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Diff_2023</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Valor_2024</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Meta_2024</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Diff_2024</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Valor_2025</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Meta_2025</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Diff_2025</t>
         </is>
@@ -584,87 +589,88 @@
       <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
         <is>
           <t>1.1 Jóvenes que acceden a servicios sociales de acuerdo con sus intereses.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes atendidos en servicios sociales para potenciar sus capacidades y mitigar sus necesidades.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Integración Social</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
       <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
         <v>0.62</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>-0.62</v>
       </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
       <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
         <v>0.63</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>-0.63</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>0.63</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>0.64</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>-0.01</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>0.78</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>0.65</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>0.13</v>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="n">
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="n">
         <v>0.66</v>
       </c>
-      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="n">
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="n">
         <v>0.67</v>
       </c>
-      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -680,93 +686,94 @@
       <c r="C3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>1.2 Jóvenes reconocidos desde sus diferentes talentos, estéticas, culturas y cosmovisiones.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que se relacionan tranquilamente con personas de culturas distintas a las suyas</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Integración Social</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.44</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.323</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>0.117</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>0.44</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>0.333</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>0.107</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>0.34</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>0.343</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>-0.003</v>
       </c>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
       <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
         <v>0.353</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>-0.353</v>
       </c>
-      <c r="W3" t="n">
-        <v>0</v>
-      </c>
       <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
         <v>0.363</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>-0.363</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>0.34</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>0.373</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>-0.033</v>
       </c>
     </row>
@@ -784,93 +791,94 @@
       <c r="C4" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>1.3 Jóvenes que participan e inciden en las dinámicas de sus territorios.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que participan en organizaciones sociales</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Gobierno</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
         <v>0.1</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>-0.1</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>0.1</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>0.105</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>-0.005</v>
       </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
       <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
         <v>0.105</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>-0.105</v>
       </c>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
       <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
         <v>0.105</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>-0.105</v>
       </c>
-      <c r="W4" t="n">
-        <v>0</v>
-      </c>
       <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
         <v>0.11</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>-0.11</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>0.02</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>0.11</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>-0.09</v>
       </c>
     </row>
@@ -888,44 +896,42 @@
       <c r="C5" t="n">
         <v>4</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>1.4 Instancias sectoriales fortalecidas para la participación juvenil.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Número de instancias sectoriales fortalecidas con participación juvenil</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Gobierno</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
@@ -933,46 +939,49 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
         <v>0.0119</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>5</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>-4.9881</v>
       </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
       <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
         <v>5</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>-5</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>2</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>5</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>-3</v>
       </c>
-      <c r="W5" t="n">
-        <v>0</v>
-      </c>
       <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
         <v>5</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>-5</v>
       </c>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="n">
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="n">
         <v>5</v>
       </c>
-      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -988,93 +997,94 @@
       <c r="C6" t="n">
         <v>5</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
         <is>
           <t>2.1 Jóvenes con acceso a educación basica secundaria que les permita proyectarse, convivir, proteger el ambiente y acceder a la ciencia y a la tecnología.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Tasa de cobertura bruta en educación básica secundaria</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>2019-01-01</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
       <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
         <v>0.924</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>-0.924</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>0.0102</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>0.924</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>-0.9137999999999999</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>1.106</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>0.924</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>0.182</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>1.0385</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>0.924</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>0.1145</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>100.58</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>0.924</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>99.65600000000001</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AA6" t="n">
         <v>102.02</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>0.924</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>101.096</v>
       </c>
     </row>
@@ -1092,93 +1102,94 @@
       <c r="C7" t="n">
         <v>6</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
         <is>
           <t>2.2 Jóvenes con acceso a educación media que les permita proyectarse, convivir, proteger el ambiente, acceder a la ciencia y a la tecnología.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Tasa de cobertura bruta en educación media</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>2019-01-01</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
       <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
         <v>0.823</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>-0.823</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>0.0051</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>0.823</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>-0.8179</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>0.978</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>0.823</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>0.155</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>0.9876</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>0.823</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>0.1646</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>0.9754</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>0.823</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>0.1524</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
         <v>101.79</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>0.823</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>100.967</v>
       </c>
     </row>
@@ -1196,93 +1207,94 @@
       <c r="C8" t="n">
         <v>7</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
         <is>
           <t>2.3 Jóvenes con acceso a educación superior que les permita proyectarse, convivir, proteger el ambiente, acceder a la ciencia y a la tecnología.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Tasa de tránsito a la educación superior</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>2019-01-01</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
       <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
         <v>0.5580000000000001</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>-0.5580000000000001</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>0.482</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>0.5580000000000001</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>-0.076</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>0.482</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0.5629999999999999</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>-0.081</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>0.515</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>0.5679999999999999</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>-0.053</v>
       </c>
-      <c r="W8" t="n">
-        <v>0</v>
-      </c>
       <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="n">
         <v>0.573</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>-0.573</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>0.5391</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>0.578</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>-0.0389</v>
       </c>
     </row>
@@ -1300,93 +1312,94 @@
       <c r="C9" t="n">
         <v>8</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
         <is>
           <t>2.4 Jóvenes que reciben educación de calidad con acceso a tecnologías de información.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Porcentaje de matrícula oficial con conexión a internet (indicador ODS conpes)</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>2019-01-01</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
       <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
         <v>1</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>-1</v>
-      </c>
-      <c r="N9" t="n">
-        <v>1</v>
       </c>
       <c r="O9" t="n">
         <v>1</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
         <v>1</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
         <v>0.9991</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>1</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>-0.0009</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>1</v>
       </c>
       <c r="AA9" t="n">
         <v>1</v>
       </c>
       <c r="AB9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1404,93 +1417,94 @@
       <c r="C10" t="n">
         <v>9</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
         <is>
           <t>2.5 Instituciones Educativas Oficiales que fomentan en los y las jóvenes prácticas para el cuidado ambiental y rural</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Porcentaje de IED Oficiales que fomentan en los jóvenes prácticas para el cuidado ambiental y rural.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>2019-01-01</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
       <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
         <v>0.32</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>-0.32</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>0.35</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>0.3216</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>0.0284</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>0.352</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>0.3216</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>0.0304</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>0.35</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>0.3216</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>0.0284</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>0.325</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>0.32</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>0.005</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AA10" t="n">
         <v>0.33</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>0.32</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -1508,93 +1522,94 @@
       <c r="C11" t="n">
         <v>10</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
         <is>
           <t>2.6. Jóvenes que cuentan con las condiciones para permanecer en la educación media .</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Tasa de deserción intranual en la educación media en el sector oficial</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>2019-01-01</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
       <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
         <v>1.53</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>-1.53</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>1.4</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>1.53</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>-0.13</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>0.006</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>1.53</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>-1.524</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>0.035</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>1.53</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>-1.495</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>0.0216</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
         <v>1.53</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>-1.5084</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AA11" t="n">
         <v>2</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>1.53</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>0.47</v>
       </c>
     </row>
@@ -1612,73 +1627,74 @@
       <c r="C12" t="n">
         <v>12</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>2.8. Jóvenes que cuentan con las condiciones para permanecer en la educación superior.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Deserción anual en programas de educación superior.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>2025-10-01</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
       <c r="V12" t="inlineStr"/>
-      <c r="W12" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
       <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="n">
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="n">
         <v>0.0949</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AB12" t="n">
         <v>0.0906</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>0.0043</v>
       </c>
     </row>
@@ -1696,93 +1712,94 @@
       <c r="C13" t="n">
         <v>13</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
         <is>
           <t>3.1. Jóvenes que acceden al mercado laboral mediante la oferta de programas de formación, vinculación y remisión a empleadores</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Jóvenes que acceden al mercado laboral a través de la Agencia Pública de Empleo</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Desarrollo Económico, Industria y Turismo</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>0.62</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>0.25</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>0.37</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>0.251</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>0.27</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>-0.019</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>0.9079</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>0.28</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>0.6279</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>0.3085</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>0.3</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>0.008500000000000001</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>0.5</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Y13" t="n">
         <v>0.31</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Z13" t="n">
         <v>0.19</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AA13" t="n">
         <v>1.17</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AB13" t="n">
         <v>0.33</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>0.84</v>
       </c>
     </row>
@@ -1800,93 +1817,94 @@
       <c r="C14" t="n">
         <v>14</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
         <is>
           <t>3.2. Jóvenes con acceso a la oferta de programas de emprendimiento, formalización, asistencia técnica y financiamiento</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que acceden a la oferta de emprendimiento, formalización, asistencia técnica y financiamiento de la SDDE</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Desarrollo Económico, Industria y Turismo</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
       <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
         <v>0.4</v>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>-0.4</v>
       </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
       <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
         <v>0.4</v>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>-0.4</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>0.13</v>
       </c>
-      <c r="R14" t="n">
+      <c r="S14" t="n">
         <v>0.4</v>
       </c>
-      <c r="S14" t="n">
+      <c r="T14" t="n">
         <v>-0.27</v>
       </c>
-      <c r="T14" t="n">
+      <c r="U14" t="n">
         <v>0.1053</v>
       </c>
-      <c r="U14" t="n">
+      <c r="V14" t="n">
         <v>0.4</v>
       </c>
-      <c r="V14" t="n">
+      <c r="W14" t="n">
         <v>-0.2947</v>
       </c>
-      <c r="W14" t="n">
+      <c r="X14" t="n">
         <v>0.172</v>
       </c>
-      <c r="X14" t="n">
+      <c r="Y14" t="n">
         <v>0.4</v>
       </c>
-      <c r="Y14" t="n">
+      <c r="Z14" t="n">
         <v>-0.228</v>
       </c>
-      <c r="Z14" t="n">
+      <c r="AA14" t="n">
         <v>0.16</v>
       </c>
-      <c r="AA14" t="n">
+      <c r="AB14" t="n">
         <v>0.4</v>
       </c>
-      <c r="AB14" t="n">
+      <c r="AC14" t="n">
         <v>-0.24</v>
       </c>
     </row>
@@ -1904,93 +1922,94 @@
       <c r="C15" t="n">
         <v>15</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
         <is>
           <t>4.1 Joven que cuenta con acceso a servicios de salud de detección temprana y protección específica en el marco de la Ruta de promoción y Mantenimiento de la Salud.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Porcentaje de personas con consulta del joven</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>0.2771</v>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>0.233</v>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>0.0441</v>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>4.94</v>
       </c>
-      <c r="O15" t="n">
+      <c r="P15" t="n">
         <v>0.252</v>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>4.688</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>0.3625</v>
       </c>
-      <c r="R15" t="n">
+      <c r="S15" t="n">
         <v>0.2663</v>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>0.09619999999999999</v>
       </c>
-      <c r="T15" t="n">
+      <c r="U15" t="n">
         <v>0.3626</v>
       </c>
-      <c r="U15" t="n">
+      <c r="V15" t="n">
         <v>0.2762</v>
       </c>
-      <c r="V15" t="n">
+      <c r="W15" t="n">
         <v>0.0864</v>
       </c>
-      <c r="W15" t="n">
+      <c r="X15" t="n">
         <v>0.3626</v>
       </c>
-      <c r="X15" t="n">
+      <c r="Y15" t="n">
         <v>0.2885</v>
       </c>
-      <c r="Y15" t="n">
+      <c r="Z15" t="n">
         <v>0.0741</v>
       </c>
-      <c r="Z15" t="n">
+      <c r="AA15" t="n">
         <v>0.3626</v>
       </c>
-      <c r="AA15" t="n">
+      <c r="AB15" t="n">
         <v>0.3008</v>
       </c>
-      <c r="AB15" t="n">
+      <c r="AC15" t="n">
         <v>0.0618</v>
       </c>
     </row>
@@ -2008,93 +2027,94 @@
       <c r="C16" t="n">
         <v>16</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
         <is>
           <t>4.2 Jóvenes que pueden identificar y prevenir riesgos en salud mental, a través de la toma de decisiones informada.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Tasa de suicidios en jóvenes</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>5.1</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>6.86</v>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>-1.76</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>4.94</v>
       </c>
-      <c r="O16" t="n">
+      <c r="P16" t="n">
         <v>7.7</v>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>-2.76</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>9.33</v>
       </c>
-      <c r="R16" t="n">
+      <c r="S16" t="n">
         <v>7.7</v>
       </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
         <v>1.63</v>
       </c>
-      <c r="T16" t="n">
+      <c r="U16" t="n">
         <v>8.66</v>
       </c>
-      <c r="U16" t="n">
+      <c r="V16" t="n">
         <v>7.7</v>
       </c>
-      <c r="V16" t="n">
+      <c r="W16" t="n">
         <v>0.96</v>
       </c>
-      <c r="W16" t="n">
+      <c r="X16" t="n">
         <v>7.5</v>
       </c>
-      <c r="X16" t="n">
+      <c r="Y16" t="n">
         <v>7.7</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Z16" t="n">
         <v>-0.2</v>
       </c>
-      <c r="Z16" t="n">
+      <c r="AA16" t="n">
         <v>6.3</v>
       </c>
-      <c r="AA16" t="n">
+      <c r="AB16" t="n">
         <v>7.7</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AC16" t="n">
         <v>-1.4</v>
       </c>
     </row>
@@ -2112,93 +2132,94 @@
       <c r="C17" t="n">
         <v>17</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
         <is>
           <t>4.3. Jóvenes que promueven estilos y hábitos de vida saludables porque cuentan con una consciencia de si, del cuidado de los demás y del ambiente.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Edad promedio de inicio de consumo abusivo de sustancias psicoactivas en población de 14 a 28 años en el Distrito Capital.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>14.9</v>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>81.77</v>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>-66.87</v>
       </c>
-      <c r="N17" t="n">
-        <v>0</v>
-      </c>
       <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
         <v>14.7</v>
       </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
         <v>-14.7</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="R17" t="n">
         <v>14.1</v>
       </c>
-      <c r="R17" t="n">
+      <c r="S17" t="n">
         <v>14.7</v>
       </c>
-      <c r="S17" t="n">
+      <c r="T17" t="n">
         <v>-0.6</v>
       </c>
-      <c r="T17" t="n">
+      <c r="U17" t="n">
         <v>14.22</v>
       </c>
-      <c r="U17" t="n">
+      <c r="V17" t="n">
         <v>14.7</v>
       </c>
-      <c r="V17" t="n">
+      <c r="W17" t="n">
         <v>-0.48</v>
       </c>
-      <c r="W17" t="n">
+      <c r="X17" t="n">
         <v>15.01</v>
       </c>
-      <c r="X17" t="n">
+      <c r="Y17" t="n">
         <v>14.7</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Z17" t="n">
         <v>0.31</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="AA17" t="n">
         <v>13.75</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AB17" t="n">
         <v>14.7</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AC17" t="n">
         <v>-0.95</v>
       </c>
     </row>
@@ -2216,93 +2237,94 @@
       <c r="C18" t="n">
         <v>18</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
         <is>
           <t>4.4. Jóvenes que toman decisiones libres frente a la maternidad y paternidad.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Tasa de fecundidad en mujeres de 15 a 19 años</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K18" t="n">
+      <c r="L18" t="n">
         <v>27.5</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>0.34</v>
       </c>
-      <c r="M18" t="n">
+      <c r="N18" t="n">
         <v>27.16</v>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>0.3005</v>
       </c>
-      <c r="O18" t="n">
+      <c r="P18" t="n">
         <v>34.6</v>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>-34.2995</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>0.2195</v>
       </c>
-      <c r="R18" t="n">
+      <c r="S18" t="n">
         <v>32.8</v>
       </c>
-      <c r="S18" t="n">
+      <c r="T18" t="n">
         <v>-32.5805</v>
       </c>
-      <c r="T18" t="n">
+      <c r="U18" t="n">
         <v>41.4</v>
       </c>
-      <c r="U18" t="n">
+      <c r="V18" t="n">
         <v>31.1</v>
       </c>
-      <c r="V18" t="n">
+      <c r="W18" t="n">
         <v>10.3</v>
       </c>
-      <c r="W18" t="n">
+      <c r="X18" t="n">
         <v>16.83</v>
       </c>
-      <c r="X18" t="n">
+      <c r="Y18" t="n">
         <v>29.5</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="Z18" t="n">
         <v>-12.67</v>
       </c>
-      <c r="Z18" t="n">
+      <c r="AA18" t="n">
         <v>16.3</v>
       </c>
-      <c r="AA18" t="n">
+      <c r="AB18" t="n">
         <v>29.5</v>
       </c>
-      <c r="AB18" t="n">
+      <c r="AC18" t="n">
         <v>-13.2</v>
       </c>
     </row>
@@ -2320,93 +2342,94 @@
       <c r="C19" t="n">
         <v>19</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
         <is>
           <t>4.5. Joven que ejerce de sus derechos sexuales y sus derechos reproductivos, de manera planeada y protegida.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Porcentaje de incidencia de VIH en jóvenes</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>84.2</v>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>86.09999999999999</v>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>-1.9</v>
       </c>
-      <c r="N19" t="n">
-        <v>0</v>
-      </c>
       <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
         <v>86.5</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>-86.5</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>102.8</v>
       </c>
-      <c r="R19" t="n">
+      <c r="S19" t="n">
         <v>87</v>
       </c>
-      <c r="S19" t="n">
+      <c r="T19" t="n">
         <v>15.8</v>
       </c>
-      <c r="T19" t="n">
+      <c r="U19" t="n">
         <v>99.3</v>
       </c>
-      <c r="U19" t="n">
+      <c r="V19" t="n">
         <v>87.40000000000001</v>
       </c>
-      <c r="V19" t="n">
+      <c r="W19" t="n">
         <v>11.9</v>
       </c>
-      <c r="W19" t="n">
+      <c r="X19" t="n">
         <v>99.09999999999999</v>
       </c>
-      <c r="X19" t="n">
+      <c r="Y19" t="n">
         <v>87.40000000000001</v>
       </c>
-      <c r="Y19" t="n">
+      <c r="Z19" t="n">
         <v>11.7</v>
       </c>
-      <c r="Z19" t="n">
+      <c r="AA19" t="n">
         <v>88.5</v>
       </c>
-      <c r="AA19" t="n">
+      <c r="AB19" t="n">
         <v>87.8</v>
       </c>
-      <c r="AB19" t="n">
+      <c r="AC19" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -2424,93 +2447,94 @@
       <c r="C20" t="n">
         <v>20</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
         <is>
           <t>5.1. Jóvenes con capacidades y espacios para poder apreciar, crear y producir bienes y servicios culturales</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que han recibido alguna formación artística</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Cultura, Recreación y Deporte</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K20" t="n">
+      <c r="L20" t="n">
         <v>0.2</v>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>9.4</v>
       </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
         <v>-9.199999999999999</v>
       </c>
-      <c r="N20" t="n">
+      <c r="O20" t="n">
         <v>0.2</v>
       </c>
-      <c r="O20" t="n">
+      <c r="P20" t="n">
         <v>0.104</v>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>0.096</v>
       </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
       <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
         <v>0.114</v>
       </c>
-      <c r="S20" t="n">
+      <c r="T20" t="n">
         <v>-0.114</v>
       </c>
-      <c r="T20" t="n">
+      <c r="U20" t="n">
         <v>0.033</v>
       </c>
-      <c r="U20" t="n">
+      <c r="V20" t="n">
         <v>0.124</v>
       </c>
-      <c r="V20" t="n">
+      <c r="W20" t="n">
         <v>-0.091</v>
       </c>
-      <c r="W20" t="n">
+      <c r="X20" t="n">
         <v>0.0675</v>
       </c>
-      <c r="X20" t="n">
+      <c r="Y20" t="n">
         <v>0.124</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="Z20" t="n">
         <v>-0.0565</v>
       </c>
-      <c r="Z20" t="n">
+      <c r="AA20" t="n">
         <v>0.0675</v>
       </c>
-      <c r="AA20" t="n">
+      <c r="AB20" t="n">
         <v>0.134</v>
       </c>
-      <c r="AB20" t="n">
+      <c r="AC20" t="n">
         <v>-0.0665</v>
       </c>
     </row>
@@ -2528,93 +2552,94 @@
       <c r="C21" t="n">
         <v>21</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
         <is>
           <t>5.2. Jóvenes con espacios artísticos, culturales y patrimoniales para participar de acuerdo con sus preferencias, tradiciones y cosmovisiones</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que realizan alguna actividad artística al mes</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Cultura, Recreación y Deporte</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K21" t="n">
+      <c r="L21" t="n">
         <v>0.18</v>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>0.323</v>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>-0.143</v>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>0.18</v>
       </c>
-      <c r="O21" t="n">
+      <c r="P21" t="n">
         <v>0.343</v>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>-0.163</v>
       </c>
-      <c r="Q21" t="n">
-        <v>0</v>
-      </c>
       <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="n">
         <v>0.363</v>
       </c>
-      <c r="S21" t="n">
+      <c r="T21" t="n">
         <v>-0.363</v>
       </c>
-      <c r="T21" t="n">
+      <c r="U21" t="n">
         <v>0.144</v>
       </c>
-      <c r="U21" t="n">
+      <c r="V21" t="n">
         <v>0.383</v>
       </c>
-      <c r="V21" t="n">
+      <c r="W21" t="n">
         <v>-0.239</v>
       </c>
-      <c r="W21" t="n">
+      <c r="X21" t="n">
         <v>0.1353</v>
       </c>
-      <c r="X21" t="n">
+      <c r="Y21" t="n">
         <v>0.383</v>
       </c>
-      <c r="Y21" t="n">
+      <c r="Z21" t="n">
         <v>-0.2477</v>
       </c>
-      <c r="Z21" t="n">
+      <c r="AA21" t="n">
         <v>0.1353</v>
       </c>
-      <c r="AA21" t="n">
+      <c r="AB21" t="n">
         <v>0.403</v>
       </c>
-      <c r="AB21" t="n">
+      <c r="AC21" t="n">
         <v>-0.2677</v>
       </c>
     </row>
@@ -2632,93 +2657,94 @@
       <c r="C22" t="n">
         <v>22</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
         <is>
           <t>5.3. Jóvenes con hábitos de lectura</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Promedio de libros leidos por jóvenes al año</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>Cultura, Recreación y Deporte</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K22" t="n">
+      <c r="L22" t="n">
         <v>1.2</v>
       </c>
-      <c r="L22" t="n">
+      <c r="M22" t="n">
         <v>5</v>
       </c>
-      <c r="M22" t="n">
+      <c r="N22" t="n">
         <v>-3.8</v>
       </c>
-      <c r="N22" t="n">
+      <c r="O22" t="n">
         <v>1.2</v>
       </c>
-      <c r="O22" t="n">
+      <c r="P22" t="n">
         <v>5</v>
       </c>
-      <c r="P22" t="n">
+      <c r="Q22" t="n">
         <v>-3.8</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="R22" t="n">
         <v>0.068</v>
       </c>
-      <c r="R22" t="n">
+      <c r="S22" t="n">
         <v>5</v>
       </c>
-      <c r="S22" t="n">
+      <c r="T22" t="n">
         <v>-4.932</v>
       </c>
-      <c r="T22" t="n">
+      <c r="U22" t="n">
         <v>6.03</v>
       </c>
-      <c r="U22" t="n">
+      <c r="V22" t="n">
         <v>5</v>
       </c>
-      <c r="V22" t="n">
+      <c r="W22" t="n">
         <v>1.03</v>
       </c>
-      <c r="W22" t="n">
+      <c r="X22" t="n">
         <v>4.4</v>
       </c>
-      <c r="X22" t="n">
+      <c r="Y22" t="n">
         <v>5</v>
       </c>
-      <c r="Y22" t="n">
+      <c r="Z22" t="n">
         <v>-0.6</v>
       </c>
-      <c r="Z22" t="n">
+      <c r="AA22" t="n">
         <v>4.4</v>
       </c>
-      <c r="AA22" t="n">
+      <c r="AB22" t="n">
         <v>6</v>
       </c>
-      <c r="AB22" t="n">
+      <c r="AC22" t="n">
         <v>-1.6</v>
       </c>
     </row>
@@ -2736,93 +2762,94 @@
       <c r="C23" t="n">
         <v>23</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
         <is>
           <t>5.4. Jóvenes satisfechos con actividades recreativas y deportivas en sus territorios.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que están satisfechos o muy satisfechos con las actividades deportivas y recreativas en su barrio</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>Cultura, Recreación y Deporte</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K23" t="n">
+      <c r="L23" t="n">
         <v>0.33</v>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>0.48</v>
       </c>
-      <c r="M23" t="n">
+      <c r="N23" t="n">
         <v>-0.15</v>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>0.33</v>
       </c>
-      <c r="O23" t="n">
+      <c r="P23" t="n">
         <v>0.55</v>
       </c>
-      <c r="P23" t="n">
+      <c r="Q23" t="n">
         <v>-0.22</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="R23" t="n">
         <v>0.5</v>
       </c>
-      <c r="R23" t="n">
+      <c r="S23" t="n">
         <v>0.58</v>
       </c>
-      <c r="S23" t="n">
+      <c r="T23" t="n">
         <v>-0.08</v>
       </c>
-      <c r="T23" t="n">
+      <c r="U23" t="n">
         <v>0.5</v>
       </c>
-      <c r="U23" t="n">
+      <c r="V23" t="n">
         <v>0.61</v>
       </c>
-      <c r="V23" t="n">
+      <c r="W23" t="n">
         <v>-0.11</v>
       </c>
-      <c r="W23" t="n">
+      <c r="X23" t="n">
         <v>0.5165</v>
       </c>
-      <c r="X23" t="n">
+      <c r="Y23" t="n">
         <v>0.61</v>
       </c>
-      <c r="Y23" t="n">
+      <c r="Z23" t="n">
         <v>-0.0935</v>
       </c>
-      <c r="Z23" t="n">
+      <c r="AA23" t="n">
         <v>0.52</v>
       </c>
-      <c r="AA23" t="n">
+      <c r="AB23" t="n">
         <v>0.64</v>
       </c>
-      <c r="AB23" t="n">
+      <c r="AC23" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -2840,93 +2867,94 @@
       <c r="C24" t="n">
         <v>24</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
         <is>
           <t>5.5. Jóvenes que realizan actividades deportivas</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que practica algún deporte.</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Cultura, Recreación y Deporte</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K24" t="n">
+      <c r="L24" t="n">
         <v>0.4</v>
       </c>
-      <c r="L24" t="n">
+      <c r="M24" t="n">
         <v>0.52</v>
       </c>
-      <c r="M24" t="n">
+      <c r="N24" t="n">
         <v>-0.12</v>
       </c>
-      <c r="N24" t="n">
+      <c r="O24" t="n">
         <v>0.4</v>
       </c>
-      <c r="O24" t="n">
+      <c r="P24" t="n">
         <v>0.54</v>
       </c>
-      <c r="P24" t="n">
+      <c r="Q24" t="n">
         <v>-0.14</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="R24" t="n">
         <v>0.41</v>
       </c>
-      <c r="R24" t="n">
+      <c r="S24" t="n">
         <v>0.55</v>
       </c>
-      <c r="S24" t="n">
+      <c r="T24" t="n">
         <v>-0.14</v>
       </c>
-      <c r="T24" t="n">
+      <c r="U24" t="n">
         <v>0.41</v>
       </c>
-      <c r="U24" t="n">
+      <c r="V24" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="V24" t="n">
+      <c r="W24" t="n">
         <v>-0.15</v>
       </c>
-      <c r="W24" t="n">
-        <v>0</v>
-      </c>
       <c r="X24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="Y24" t="n">
+      <c r="Z24" t="n">
         <v>-0.5600000000000001</v>
       </c>
-      <c r="Z24" t="n">
+      <c r="AA24" t="n">
         <v>0.41</v>
       </c>
-      <c r="AA24" t="n">
+      <c r="AB24" t="n">
         <v>0.57</v>
       </c>
-      <c r="AB24" t="n">
+      <c r="AC24" t="n">
         <v>-0.16</v>
       </c>
     </row>
@@ -2944,91 +2972,92 @@
       <c r="C25" t="n">
         <v>25</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
         <is>
           <t>6.1 Jóvenes que cuentan con entornos seguros que favorecen su integridad personal.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Tasa de lesiones personales en jóvenes 18-28 años por cada 100.000 habitantes de jóvenes entre los 18-28 años</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Seguridad, Convivencia y Justicia</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
       <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
         <v>473.5</v>
       </c>
-      <c r="M25" t="n">
+      <c r="N25" t="n">
         <v>-473.5</v>
       </c>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
       <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
         <v>459.5</v>
       </c>
-      <c r="P25" t="n">
+      <c r="Q25" t="n">
         <v>-459.5</v>
       </c>
-      <c r="Q25" t="n">
-        <v>0</v>
-      </c>
       <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
         <v>452.5</v>
       </c>
-      <c r="S25" t="n">
+      <c r="T25" t="n">
         <v>-452.5</v>
       </c>
-      <c r="T25" t="n">
-        <v>0</v>
-      </c>
       <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
         <v>445.5</v>
       </c>
-      <c r="V25" t="n">
+      <c r="W25" t="n">
         <v>-445.5</v>
       </c>
-      <c r="W25" t="n">
+      <c r="X25" t="n">
         <v>333</v>
       </c>
-      <c r="X25" t="n">
+      <c r="Y25" t="n">
         <v>445.5</v>
       </c>
-      <c r="Y25" t="n">
+      <c r="Z25" t="n">
         <v>-112.5</v>
       </c>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="n">
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="n">
         <v>438.5</v>
       </c>
-      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3044,91 +3073,92 @@
       <c r="C26" t="n">
         <v>26</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
         <is>
           <t>6.2. Jóvenes que cuentan con entornos seguros y libres de riesgos y amenzas de vinculación o instrumentalización.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Tasa por 100.000 habitantes de jóvenes entre los 14 y 17 años en el SRPA</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>Seguridad, Convivencia y Justicia</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
       <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
         <v>1079</v>
       </c>
-      <c r="M26" t="n">
+      <c r="N26" t="n">
         <v>-1079</v>
       </c>
-      <c r="N26" t="n">
-        <v>0</v>
-      </c>
       <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
         <v>1062.2569</v>
       </c>
-      <c r="P26" t="n">
+      <c r="Q26" t="n">
         <v>-1062.2569</v>
       </c>
-      <c r="Q26" t="n">
-        <v>0</v>
-      </c>
       <c r="R26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" t="n">
         <v>1045.8303</v>
       </c>
-      <c r="S26" t="n">
+      <c r="T26" t="n">
         <v>-1045.8303</v>
       </c>
-      <c r="T26" t="n">
-        <v>0</v>
-      </c>
       <c r="U26" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" t="n">
         <v>1029.4036</v>
       </c>
-      <c r="V26" t="n">
+      <c r="W26" t="n">
         <v>-1029.4036</v>
       </c>
-      <c r="W26" t="n">
-        <v>0</v>
-      </c>
       <c r="X26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" t="n">
         <v>1029</v>
       </c>
-      <c r="Y26" t="n">
+      <c r="Z26" t="n">
         <v>-1029</v>
       </c>
-      <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="n">
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="n">
         <v>1013</v>
       </c>
-      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3144,93 +3174,94 @@
       <c r="C27" t="n">
         <v>27</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
         <is>
           <t>6.3. Jóvenes con entornos familiares seguros</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Tasa de violencia intrafamiliar</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>Integración Social</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
       <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
         <v>242</v>
       </c>
-      <c r="M27" t="n">
+      <c r="N27" t="n">
         <v>-242</v>
       </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
       <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
         <v>235</v>
       </c>
-      <c r="P27" t="n">
+      <c r="Q27" t="n">
         <v>-235</v>
       </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
       <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
         <v>229</v>
       </c>
-      <c r="S27" t="n">
+      <c r="T27" t="n">
         <v>-229</v>
       </c>
-      <c r="T27" t="n">
-        <v>0</v>
-      </c>
       <c r="U27" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" t="n">
         <v>223</v>
       </c>
-      <c r="V27" t="n">
+      <c r="W27" t="n">
         <v>-223</v>
       </c>
-      <c r="W27" t="n">
+      <c r="X27" t="n">
         <v>84</v>
       </c>
-      <c r="X27" t="n">
+      <c r="Y27" t="n">
         <v>223</v>
       </c>
-      <c r="Y27" t="n">
+      <c r="Z27" t="n">
         <v>-139</v>
       </c>
-      <c r="Z27" t="n">
+      <c r="AA27" t="n">
         <v>331</v>
       </c>
-      <c r="AA27" t="n">
+      <c r="AB27" t="n">
         <v>218</v>
       </c>
-      <c r="AB27" t="n">
+      <c r="AC27" t="n">
         <v>113</v>
       </c>
     </row>
@@ -3248,93 +3279,94 @@
       <c r="C28" t="n">
         <v>28</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
         <is>
           <t>6.4. Jóvenes que cuentan con entornos seguros sin riesgos y amenazas de explotación y trata.</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Tasa de trata de personas en jóvenes entre 18- 28 años</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>Gobierno</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K28" t="n">
+      <c r="L28" t="n">
         <v>0.4</v>
       </c>
-      <c r="L28" t="n">
+      <c r="M28" t="n">
         <v>0.9999</v>
       </c>
-      <c r="M28" t="n">
+      <c r="N28" t="n">
         <v>-0.5999</v>
       </c>
-      <c r="N28" t="n">
+      <c r="O28" t="n">
         <v>0.51</v>
       </c>
-      <c r="O28" t="n">
+      <c r="P28" t="n">
         <v>0.9998</v>
       </c>
-      <c r="P28" t="n">
+      <c r="Q28" t="n">
         <v>-0.4898</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="R28" t="n">
         <v>1.1</v>
       </c>
-      <c r="R28" t="n">
+      <c r="S28" t="n">
         <v>0.9997</v>
       </c>
-      <c r="S28" t="n">
+      <c r="T28" t="n">
         <v>0.1003</v>
       </c>
-      <c r="T28" t="n">
+      <c r="U28" t="n">
         <v>1.62</v>
       </c>
-      <c r="U28" t="n">
+      <c r="V28" t="n">
         <v>0.9996</v>
       </c>
-      <c r="V28" t="n">
+      <c r="W28" t="n">
         <v>0.6204</v>
       </c>
-      <c r="W28" t="n">
-        <v>0</v>
-      </c>
       <c r="X28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" t="n">
         <v>0.9995000000000001</v>
       </c>
-      <c r="Y28" t="n">
+      <c r="Z28" t="n">
         <v>-0.9995000000000001</v>
       </c>
-      <c r="Z28" t="n">
+      <c r="AA28" t="n">
         <v>3.0612</v>
       </c>
-      <c r="AA28" t="n">
+      <c r="AB28" t="n">
         <v>0.9994</v>
       </c>
-      <c r="AB28" t="n">
+      <c r="AC28" t="n">
         <v>2.0618</v>
       </c>
     </row>
@@ -3352,93 +3384,94 @@
       <c r="C29" t="n">
         <v>29</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
         <is>
           <t>6.5. Jóvenes que cuentan con entornos seguros para el ejercicio de su ciudadanía</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Tasa de desaparición forzosa en persona (art. 166 CP, art. 4)</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>Gobierno</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K29" t="n">
+      <c r="L29" t="n">
         <v>0.4</v>
       </c>
-      <c r="L29" t="n">
+      <c r="M29" t="n">
         <v>0.0109</v>
       </c>
-      <c r="M29" t="n">
+      <c r="N29" t="n">
         <v>0.3891</v>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>0.82</v>
       </c>
-      <c r="O29" t="n">
+      <c r="P29" t="n">
         <v>0.0109</v>
       </c>
-      <c r="P29" t="n">
+      <c r="Q29" t="n">
         <v>0.8091</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="R29" t="n">
         <v>3.04</v>
       </c>
-      <c r="R29" t="n">
+      <c r="S29" t="n">
         <v>0.0108</v>
       </c>
-      <c r="S29" t="n">
+      <c r="T29" t="n">
         <v>3.0292</v>
       </c>
-      <c r="T29" t="n">
+      <c r="U29" t="n">
         <v>3.83</v>
       </c>
-      <c r="U29" t="n">
+      <c r="V29" t="n">
         <v>0.0107</v>
       </c>
-      <c r="V29" t="n">
+      <c r="W29" t="n">
         <v>3.8193</v>
       </c>
-      <c r="W29" t="n">
-        <v>0</v>
-      </c>
       <c r="X29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" t="n">
         <v>0.0107</v>
       </c>
-      <c r="Y29" t="n">
+      <c r="Z29" t="n">
         <v>-0.0107</v>
       </c>
-      <c r="Z29" t="n">
+      <c r="AA29" t="n">
         <v>4.66</v>
       </c>
-      <c r="AA29" t="n">
+      <c r="AB29" t="n">
         <v>0.0106</v>
       </c>
-      <c r="AB29" t="n">
+      <c r="AC29" t="n">
         <v>4.6494</v>
       </c>
     </row>
@@ -3456,91 +3489,92 @@
       <c r="C30" t="n">
         <v>30</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
         <is>
           <t>6.6. Jóvenes con oportunidades y herramientas para conciliar ante situaciones de conflicto en los territorios.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que perciben el espacio público como peligroso o conflictivo</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>Seguridad, Convivencia y Justicia</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
       <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
         <v>0.8863</v>
       </c>
-      <c r="M30" t="n">
+      <c r="N30" t="n">
         <v>-0.8863</v>
       </c>
-      <c r="N30" t="n">
-        <v>0</v>
-      </c>
       <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
         <v>0.8763</v>
       </c>
-      <c r="P30" t="n">
+      <c r="Q30" t="n">
         <v>-0.8763</v>
       </c>
-      <c r="Q30" t="n">
-        <v>0</v>
-      </c>
       <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
         <v>0.8663</v>
       </c>
-      <c r="S30" t="n">
+      <c r="T30" t="n">
         <v>-0.8663</v>
       </c>
-      <c r="T30" t="n">
-        <v>0</v>
-      </c>
       <c r="U30" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
         <v>0.8563</v>
       </c>
-      <c r="V30" t="n">
+      <c r="W30" t="n">
         <v>-0.8563</v>
       </c>
-      <c r="W30" t="n">
-        <v>0</v>
-      </c>
       <c r="X30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" t="n">
         <v>0.8563</v>
       </c>
-      <c r="Y30" t="n">
+      <c r="Z30" t="n">
         <v>-0.8563</v>
       </c>
-      <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="n">
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="n">
         <v>0.8463000000000001</v>
       </c>
-      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3556,93 +3590,94 @@
       <c r="C31" t="n">
         <v>31</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
         <is>
           <t>6.7. Jóvenes comprometidos con la construcción de paz y reconciliación.</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que consideran que las actividades realizadas profundizan su compromiso en la memoria, paz y reconciliación</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>Gestión Pública</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
       <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
         <v>0.7</v>
       </c>
-      <c r="M31" t="n">
+      <c r="N31" t="n">
         <v>-0.7</v>
       </c>
-      <c r="N31" t="n">
-        <v>0</v>
-      </c>
       <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
         <v>0.7</v>
       </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
         <v>-0.7</v>
       </c>
-      <c r="Q31" t="n">
-        <v>0</v>
-      </c>
       <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
         <v>0.7</v>
       </c>
-      <c r="S31" t="n">
+      <c r="T31" t="n">
         <v>-0.7</v>
-      </c>
-      <c r="T31" t="n">
-        <v>0.7</v>
       </c>
       <c r="U31" t="n">
         <v>0.7</v>
       </c>
       <c r="V31" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="W31" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" t="n">
         <v>1</v>
       </c>
-      <c r="X31" t="n">
+      <c r="Y31" t="n">
         <v>0.7</v>
       </c>
-      <c r="Y31" t="n">
+      <c r="Z31" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z31" t="n">
+      <c r="AA31" t="n">
         <v>0.98</v>
       </c>
-      <c r="AA31" t="n">
+      <c r="AB31" t="n">
         <v>0.7</v>
       </c>
-      <c r="AB31" t="n">
+      <c r="AC31" t="n">
         <v>0.28</v>
       </c>
     </row>
@@ -3660,91 +3695,92 @@
       <c r="C32" t="n">
         <v>32</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
         <is>
           <t>6.8. Jóvenes vinculados a procesos penales capaces de planear sus proyectos de vida basados en la cultura de la legalidad</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Porcentaje de reincidentes condenados de 18 a 28 años en las cárceles nacionales</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>Seguridad, Convivencia y Justicia</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
       <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
         <v>0.1919</v>
       </c>
-      <c r="M32" t="n">
+      <c r="N32" t="n">
         <v>-0.1919</v>
       </c>
-      <c r="N32" t="n">
-        <v>0</v>
-      </c>
       <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
         <v>0.1908</v>
       </c>
-      <c r="P32" t="n">
+      <c r="Q32" t="n">
         <v>-0.1908</v>
       </c>
-      <c r="Q32" t="n">
-        <v>0</v>
-      </c>
       <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
         <v>0.1897</v>
       </c>
-      <c r="S32" t="n">
+      <c r="T32" t="n">
         <v>-0.1897</v>
       </c>
-      <c r="T32" t="n">
-        <v>0</v>
-      </c>
       <c r="U32" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" t="n">
         <v>0.1886</v>
       </c>
-      <c r="V32" t="n">
+      <c r="W32" t="n">
         <v>-0.1886</v>
       </c>
-      <c r="W32" t="n">
-        <v>0</v>
-      </c>
       <c r="X32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" t="n">
         <v>0.1886</v>
       </c>
-      <c r="Y32" t="n">
+      <c r="Z32" t="n">
         <v>-0.1886</v>
       </c>
-      <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="n">
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="n">
         <v>0.1875</v>
       </c>
-      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3760,93 +3796,94 @@
       <c r="C33" t="n">
         <v>33</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
         <is>
           <t>7.1. Jóvenes con consciencia ambiental y con la capacidad de entender la incidencia de sus acciones cotidianas sobre el ambiente de la Ciudad y la región.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que realizan alguna práctica de reciclaje</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K33" t="n">
+      <c r="L33" t="n">
         <v>0.1005</v>
       </c>
-      <c r="L33" t="n">
+      <c r="M33" t="n">
         <v>0.613</v>
       </c>
-      <c r="M33" t="n">
+      <c r="N33" t="n">
         <v>-0.5125</v>
       </c>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
       <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
         <v>0.6145</v>
       </c>
-      <c r="P33" t="n">
+      <c r="Q33" t="n">
         <v>-0.6145</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="R33" t="n">
         <v>0.2525</v>
       </c>
-      <c r="R33" t="n">
+      <c r="S33" t="n">
         <v>0.616</v>
       </c>
-      <c r="S33" t="n">
+      <c r="T33" t="n">
         <v>-0.3635</v>
       </c>
-      <c r="T33" t="n">
+      <c r="U33" t="n">
         <v>0.98</v>
       </c>
-      <c r="U33" t="n">
+      <c r="V33" t="n">
         <v>0.6175</v>
       </c>
-      <c r="V33" t="n">
+      <c r="W33" t="n">
         <v>0.3625</v>
       </c>
-      <c r="W33" t="n">
+      <c r="X33" t="n">
         <v>0.99</v>
       </c>
-      <c r="X33" t="n">
+      <c r="Y33" t="n">
         <v>0.6175</v>
       </c>
-      <c r="Y33" t="n">
+      <c r="Z33" t="n">
         <v>0.3725</v>
       </c>
-      <c r="Z33" t="n">
+      <c r="AA33" t="n">
         <v>0.99</v>
       </c>
-      <c r="AA33" t="n">
+      <c r="AB33" t="n">
         <v>0.619</v>
       </c>
-      <c r="AB33" t="n">
+      <c r="AC33" t="n">
         <v>0.371</v>
       </c>
     </row>
@@ -3864,87 +3901,88 @@
       <c r="C34" t="n">
         <v>34</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
         <is>
           <t>7.2. Jóvenes que protegen y fomentan el bienestar animal.</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que se vinculan a procesos de movilización social por la protección y el bienestar animal</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>Ambiente</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K34" t="n">
+      <c r="L34" t="n">
         <v>0.2354</v>
       </c>
-      <c r="L34" t="n">
+      <c r="M34" t="n">
         <v>0.45</v>
       </c>
-      <c r="M34" t="n">
+      <c r="N34" t="n">
         <v>-0.2146</v>
       </c>
-      <c r="N34" t="n">
+      <c r="O34" t="n">
         <v>0.4079</v>
       </c>
-      <c r="O34" t="n">
+      <c r="P34" t="n">
         <v>0.47</v>
       </c>
-      <c r="P34" t="n">
+      <c r="Q34" t="n">
         <v>-0.0621</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="R34" t="n">
         <v>1</v>
       </c>
-      <c r="R34" t="n">
+      <c r="S34" t="n">
         <v>0.48</v>
       </c>
-      <c r="S34" t="n">
+      <c r="T34" t="n">
         <v>0.52</v>
       </c>
-      <c r="T34" t="n">
+      <c r="U34" t="n">
         <v>1</v>
       </c>
-      <c r="U34" t="n">
+      <c r="V34" t="n">
         <v>0.49</v>
       </c>
-      <c r="V34" t="n">
+      <c r="W34" t="n">
         <v>0.51</v>
       </c>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="n">
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="n">
         <v>0.48</v>
       </c>
-      <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="inlineStr"/>
-      <c r="AA34" t="n">
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="n">
         <v>0.49</v>
       </c>
-      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3960,93 +3998,94 @@
       <c r="C35" t="n">
         <v>35</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
         <is>
           <t>7.3. Jóvenes que habitan en una vivienda digna.</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que viven en una vivienda sin deficit habitacional</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>Hábitat</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K35" t="n">
+      <c r="L35" t="n">
         <v>1</v>
       </c>
-      <c r="L35" t="n">
+      <c r="M35" t="n">
         <v>0.951</v>
       </c>
-      <c r="M35" t="n">
+      <c r="N35" t="n">
         <v>0.049</v>
       </c>
-      <c r="N35" t="n">
+      <c r="O35" t="n">
         <v>1</v>
       </c>
-      <c r="O35" t="n">
+      <c r="P35" t="n">
         <v>0.954</v>
       </c>
-      <c r="P35" t="n">
+      <c r="Q35" t="n">
         <v>0.046</v>
       </c>
-      <c r="Q35" t="n">
-        <v>0</v>
-      </c>
       <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="n">
         <v>0.957</v>
       </c>
-      <c r="S35" t="n">
+      <c r="T35" t="n">
         <v>-0.957</v>
       </c>
-      <c r="T35" t="n">
-        <v>0</v>
-      </c>
       <c r="U35" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
         <v>0.96</v>
       </c>
-      <c r="V35" t="n">
+      <c r="W35" t="n">
         <v>-0.96</v>
       </c>
-      <c r="W35" t="n">
-        <v>0</v>
-      </c>
       <c r="X35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" t="n">
         <v>0.957</v>
       </c>
-      <c r="Y35" t="n">
+      <c r="Z35" t="n">
         <v>-0.957</v>
       </c>
-      <c r="Z35" t="n">
+      <c r="AA35" t="n">
         <v>0.84</v>
       </c>
-      <c r="AA35" t="n">
+      <c r="AB35" t="n">
         <v>0.96</v>
       </c>
-      <c r="AB35" t="n">
+      <c r="AC35" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -4064,93 +4103,94 @@
       <c r="C36" t="n">
         <v>36</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
         <is>
           <t>7.4. Jóvenes que se movilizan en transportes amigables o ambientalmente sostenibles.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Porcentaje de jóvenes que se movilizan principalmente caminando o en bicicleta</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Porcentaje</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>Creciente</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K36" t="n">
-        <v>0</v>
-      </c>
       <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
         <v>0.32</v>
       </c>
-      <c r="M36" t="n">
+      <c r="N36" t="n">
         <v>-0.32</v>
       </c>
-      <c r="N36" t="n">
+      <c r="O36" t="n">
         <v>0.18</v>
       </c>
-      <c r="O36" t="n">
+      <c r="P36" t="n">
         <v>0.335</v>
       </c>
-      <c r="P36" t="n">
+      <c r="Q36" t="n">
         <v>-0.155</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="R36" t="n">
         <v>0.18</v>
       </c>
-      <c r="R36" t="n">
+      <c r="S36" t="n">
         <v>0.35</v>
       </c>
-      <c r="S36" t="n">
+      <c r="T36" t="n">
         <v>-0.17</v>
       </c>
-      <c r="T36" t="n">
-        <v>0</v>
-      </c>
       <c r="U36" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" t="n">
         <v>0.365</v>
       </c>
-      <c r="V36" t="n">
+      <c r="W36" t="n">
         <v>-0.365</v>
       </c>
-      <c r="W36" t="n">
+      <c r="X36" t="n">
         <v>0.18</v>
       </c>
-      <c r="X36" t="n">
+      <c r="Y36" t="n">
         <v>0.35</v>
       </c>
-      <c r="Y36" t="n">
+      <c r="Z36" t="n">
         <v>-0.17</v>
       </c>
-      <c r="Z36" t="n">
-        <v>0</v>
-      </c>
       <c r="AA36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB36" t="n">
         <v>0.365</v>
       </c>
-      <c r="AB36" t="n">
+      <c r="AC36" t="n">
         <v>-0.365</v>
       </c>
     </row>
@@ -4168,93 +4208,94 @@
       <c r="C37" t="n">
         <v>37</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
         <is>
           <t>7.5. Jóvenes que se movilizan de manera segura en la ciudad</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Tasa de mortalidad por accidentes de tránsito en jóvenes de 15 a 29 años</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Tasa</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>Decreciente</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="K37" t="n">
+      <c r="L37" t="n">
         <v>142</v>
       </c>
-      <c r="L37" t="n">
+      <c r="M37" t="n">
         <v>7.38</v>
       </c>
-      <c r="M37" t="n">
+      <c r="N37" t="n">
         <v>134.62</v>
       </c>
-      <c r="N37" t="n">
+      <c r="O37" t="n">
         <v>0.0827</v>
       </c>
-      <c r="O37" t="n">
+      <c r="P37" t="n">
         <v>6.9925</v>
       </c>
-      <c r="P37" t="n">
+      <c r="Q37" t="n">
         <v>-6.9098</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="R37" t="n">
         <v>0.0827</v>
       </c>
-      <c r="R37" t="n">
+      <c r="S37" t="n">
         <v>6.6123</v>
       </c>
-      <c r="S37" t="n">
+      <c r="T37" t="n">
         <v>-6.5296</v>
       </c>
-      <c r="T37" t="n">
+      <c r="U37" t="n">
         <v>10.32</v>
       </c>
-      <c r="U37" t="n">
+      <c r="V37" t="n">
         <v>6.2823</v>
       </c>
-      <c r="V37" t="n">
+      <c r="W37" t="n">
         <v>4.0377</v>
       </c>
-      <c r="W37" t="n">
+      <c r="X37" t="n">
         <v>11.1</v>
       </c>
-      <c r="X37" t="n">
+      <c r="Y37" t="n">
         <v>6.61</v>
       </c>
-      <c r="Y37" t="n">
+      <c r="Z37" t="n">
         <v>4.49</v>
       </c>
-      <c r="Z37" t="n">
+      <c r="AA37" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="AA37" t="n">
+      <c r="AB37" t="n">
         <v>6.28</v>
       </c>
-      <c r="AB37" t="n">
+      <c r="AC37" t="n">
         <v>2.92</v>
       </c>
     </row>

</xml_diff>